<commit_message>
in vivo analysis and primer design
</commit_message>
<xml_diff>
--- a/source_data/10_validation_guides/CDK2_4_6_validation_guides.xlsx
+++ b/source_data/10_validation_guides/CDK2_4_6_validation_guides.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samgould/Documents/GitHub/CDK-BE-mutagenesis/source_data/10_validation_guides/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BE91149-676D-5545-8B2A-143EDAF7BFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD19A7F-FF0C-CC43-8AA2-3B062D903B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -477,26 +477,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,16 +828,16 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="4" t="s">
         <v>104</v>
       </c>
     </row>
@@ -857,7 +858,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <f>RIGHT(B2, 20)</f>
+        <f t="shared" ref="G2:G15" si="0">RIGHT(B2, 20)</f>
         <v>GCTGCTTATTAACACAGAGG</v>
       </c>
       <c r="H2" t="s">
@@ -885,7 +886,7 @@
         <v>2</v>
       </c>
       <c r="G3" t="str">
-        <f>RIGHT(B3, 20)</f>
+        <f t="shared" si="0"/>
         <v>GTTAAGCTCCTTAAGCAGAG</v>
       </c>
       <c r="H3" t="s">
@@ -913,14 +914,14 @@
         <v>3</v>
       </c>
       <c r="G4" t="str">
-        <f>RIGHT(B4, 20)</f>
+        <f t="shared" si="0"/>
         <v>GAAATTCAAAAACCAGGTAG</v>
       </c>
       <c r="H4" t="s">
         <v>107</v>
       </c>
       <c r="I4" t="b">
-        <f t="shared" ref="I4:I15" si="0">G4=H4</f>
+        <f t="shared" ref="I4:I15" si="1">G4=H4</f>
         <v>1</v>
       </c>
     </row>
@@ -941,14 +942,14 @@
         <v>4</v>
       </c>
       <c r="G5" t="str">
-        <f>RIGHT(B5, 20)</f>
+        <f t="shared" si="0"/>
         <v>GAGAAATTCAAAAACCAGGT</v>
       </c>
       <c r="H5" t="s">
         <v>108</v>
       </c>
       <c r="I5" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -969,14 +970,14 @@
         <v>5</v>
       </c>
       <c r="G6" t="str">
-        <f>RIGHT(B6, 20)</f>
+        <f t="shared" si="0"/>
         <v>GCTCTGGCTAGTCCAAAGTC</v>
       </c>
       <c r="H6" t="s">
         <v>119</v>
       </c>
       <c r="I6" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -997,14 +998,14 @@
         <v>7</v>
       </c>
       <c r="G7" t="str">
-        <f>RIGHT(B7, 20)</f>
+        <f t="shared" si="0"/>
         <v>GTTGTCACCAGAATGTTCTC</v>
       </c>
       <c r="H7" t="s">
         <v>110</v>
       </c>
       <c r="I7" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1025,14 +1026,14 @@
         <v>6</v>
       </c>
       <c r="G8" t="str">
-        <f>RIGHT(B8, 20)</f>
+        <f t="shared" si="0"/>
         <v>GCCTCACGAACTGTGCTGAT</v>
       </c>
       <c r="H8" t="s">
         <v>109</v>
       </c>
       <c r="I8" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1053,14 +1054,14 @@
         <v>8</v>
       </c>
       <c r="G9" t="str">
-        <f>RIGHT(B9, 20)</f>
+        <f t="shared" si="0"/>
         <v>GTGCCAATTGCATCGTTCAC</v>
       </c>
       <c r="H9" t="s">
         <v>111</v>
       </c>
       <c r="I9" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1081,14 +1082,14 @@
         <v>9</v>
       </c>
       <c r="G10" t="str">
-        <f>RIGHT(B10, 20)</f>
+        <f t="shared" si="0"/>
         <v>GGCATGTAGACCAGGACCTA</v>
       </c>
       <c r="H10" t="s">
         <v>112</v>
       </c>
       <c r="I10" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1109,14 +1110,14 @@
         <v>10</v>
       </c>
       <c r="G11" t="str">
-        <f>RIGHT(B11, 20)</f>
+        <f t="shared" si="0"/>
         <v>GCCTTCCCATCAGCACAGTT</v>
       </c>
       <c r="H11" t="s">
         <v>113</v>
       </c>
       <c r="I11" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1137,14 +1138,14 @@
         <v>11</v>
       </c>
       <c r="G12" t="str">
-        <f>RIGHT(B12, 20)</f>
+        <f t="shared" si="0"/>
         <v>GGGTCAAGTCTTGATCGACA</v>
       </c>
       <c r="H12" t="s">
         <v>114</v>
       </c>
       <c r="I12" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1165,14 +1166,14 @@
         <v>12</v>
       </c>
       <c r="G13" t="str">
-        <f>RIGHT(B13, 20)</f>
+        <f t="shared" si="0"/>
         <v>GAGCGGCATGCCCTCCTCGC</v>
       </c>
       <c r="H13" t="s">
         <v>116</v>
       </c>
       <c r="I13" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1193,14 +1194,14 @@
         <v>13</v>
       </c>
       <c r="G14" t="str">
-        <f>RIGHT(B14, 20)</f>
+        <f t="shared" si="0"/>
         <v>GGCCTCCGTTCTTCAAGTCG</v>
       </c>
       <c r="H14" t="s">
         <v>117</v>
       </c>
       <c r="I14" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1221,14 +1222,14 @@
         <v>14</v>
       </c>
       <c r="G15" t="str">
-        <f>RIGHT(B15, 20)</f>
+        <f t="shared" si="0"/>
         <v>GGGGAGGGCGCCTATGGGAA</v>
       </c>
       <c r="H15" t="s">
         <v>118</v>
       </c>
       <c r="I15" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -1439,323 +1440,323 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" customWidth="1"/>
+    <col min="1" max="1" width="3.5" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="4" max="4" width="8.1640625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="7.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="9">
         <v>54.302554000000001</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="9">
         <v>37.007700999999997</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="9">
         <v>34.814577999999997</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="A5" s="6">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="9">
         <v>39.735894000000002</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6">
+    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="9">
         <v>25.903254</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="A7" s="6">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="9">
         <v>41.541404</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="9">
         <v>71.254019</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="9">
         <v>69.879855000000006</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="A10" s="6">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="9">
         <v>33.375985</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11">
+    <row r="11" spans="1:7" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="9">
         <v>39.518351000000003</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="9">
         <v>23.940639999999998</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="9" t="s">
         <v>71</v>
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13">
+    <row r="13" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="6">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="9">
         <v>19.351908000000002</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14">
+      <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="9">
         <v>32.186906999999998</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15">
+      <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="9">
         <v>50.834201999999998</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G15" s="2"/>

</xml_diff>